<commit_message>
feat: Production-grade SQL validation project completed with full functionality and professional reporting
</commit_message>
<xml_diff>
--- a/reports/SUMMARY_REPORT.xlsx
+++ b/reports/SUMMARY_REPORT.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Issue Details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Recommendations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,29 +427,267 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Reports Generated</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>All critical validation checks completed</t>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SQL Test Data Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chinook</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Checks Performed</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Total Issues Found</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Issues Detected</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Issues Found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>high_value_invoices</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>invoices_negative_total</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>invoices_per_customer</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>invoices_without_lines</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>invoices_without_valid_customer</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>invoices_zero_items</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>invoice_date_future</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>invoice_total_mismatch</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>negative_quantity</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>total_customers</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>zero_price_items</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fix any duplicate emails if found</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Enforce NOT NULL on required customer fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Validate email format on data insert/update</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Add check constraints for positive totals/quantities/prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ensure every invoice has at least one line item</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>